<commit_message>
fix: update contract payment status logic and improve date handling
</commit_message>
<xml_diff>
--- a/CURRETN_SHEETS_STATE.xlsx
+++ b/CURRETN_SHEETS_STATE.xlsx
@@ -25,10 +25,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={64c36c4f-179b-47d1-bffa-a0175fb360c5}</author>
+    <author>tc={7438e2bf-8da9-4a3d-a9a1-5183d8e4e61c}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{64c36c4f-179b-47d1-bffa-a0175fb360c5}" ref="G1">
+    <comment authorId="0" xr:uid="{7438e2bf-8da9-4a3d-a9a1-5183d8e4e61c}" ref="G1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="315">
   <si>
     <t>Project ID</t>
   </si>
@@ -777,6 +777,9 @@
     <t>Rough works</t>
   </si>
   <si>
+    <t>Completed</t>
+  </si>
+  <si>
     <t>D2</t>
   </si>
   <si>
@@ -787,6 +790,9 @@
   </si>
   <si>
     <t>Facade</t>
+  </si>
+  <si>
+    <t>Active</t>
   </si>
   <si>
     <t>Expense ID</t>
@@ -1765,11 +1771,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1156861237"/>
-        <c:axId val="627923265"/>
+        <c:axId val="1537677334"/>
+        <c:axId val="811568496"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1156861237"/>
+        <c:axId val="1537677334"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1821,10 +1827,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="627923265"/>
+        <c:crossAx val="811568496"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="627923265"/>
+        <c:axId val="811568496"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1899,7 +1905,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1156861237"/>
+        <c:crossAx val="1537677334"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2079,7 +2085,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Magomed Omarov (alkihuri)" id="{fa1c9bdb-908c-4985-9d54-f1034588ed56}" providerId="google-sheets"/>
+  <x18tc:person displayName="Magomed Omarov (alkihuri)" id="{276639bb-e941-47c4-a3f9-b5a7fa74a59b}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -2490,7 +2496,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="G1" dT="2026-04-23T13:21:18.00" personId="{fa1c9bdb-908c-4985-9d54-f1034588ed56}" id="{64c36c4f-179b-47d1-bffa-a0175fb360c5}" done="0">
+  <x18tc:threadedComment ref="G1" dT="2026-04-23T13:21:18.00" personId="{276639bb-e941-47c4-a3f9-b5a7fa74a59b}" id="{7438e2bf-8da9-4a3d-a9a1-5183d8e4e61c}" done="0">
     <x18tc:text xml:space="preserve">Тут просто верификация расчетов</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -2802,42 +2808,42 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>66</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E2" s="32">
         <v>350000.0</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1"/>
@@ -2877,25 +2883,25 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="G1" s="41" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
@@ -3094,22 +3100,22 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="62" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B1" s="62" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="63" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D1" s="62" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E1" s="62" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="F1" s="62" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="G1" s="64" t="s">
         <v>19</v>
@@ -3135,7 +3141,7 @@
         <v>2603305.785123967</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
@@ -3158,7 +3164,7 @@
         <v>4338842.975206612</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
@@ -3181,7 +3187,7 @@
         <v>4252066.115702479</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
@@ -3204,7 +3210,7 @@
         <v>9458677.685950413</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
@@ -3227,7 +3233,7 @@
         <v>9979338.842975207</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -3250,7 +3256,7 @@
         <v>1.0152892561983472E7</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
@@ -3273,7 +3279,7 @@
         <v>1.05E7</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
@@ -3296,7 +3302,7 @@
         <v>1.0479173553719008E7</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
@@ -3319,7 +3325,7 @@
         <v>1.0652727272727273E7</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
@@ -3342,7 +3348,7 @@
         <v>9906446.280991737</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
@@ -3365,7 +3371,7 @@
         <v>1.0080000000000002E7</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
@@ -3388,7 +3394,7 @@
         <v>1.042710743801653E7</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
@@ -3411,7 +3417,7 @@
         <v>1.0947768595041323E7</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
@@ -3434,7 +3440,7 @@
         <v>1.120809917355372E7</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
@@ -3457,7 +3463,7 @@
         <v>1.1468429752066117E7</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
@@ -3480,7 +3486,7 @@
         <v>1.1641983471074382E7</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
@@ -3503,7 +3509,7 @@
         <v>1.2162644628099175E7</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19">
@@ -6484,13 +6490,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="67" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B1" s="68"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B2" s="2">
         <v>3.0</v>
@@ -6498,7 +6504,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B3" s="2">
         <v>2.0</v>
@@ -6506,7 +6512,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B4" s="2">
         <v>0.0</v>
@@ -6514,13 +6520,13 @@
     </row>
     <row r="6">
       <c r="A6" s="67" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B6" s="69"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B7" s="2">
         <v>605000.0</v>
@@ -6528,7 +6534,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B8" s="2">
         <v>7.5E7</v>
@@ -6536,7 +6542,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B9" s="2">
         <v>-7.4395E7</v>
@@ -6544,43 +6550,43 @@
     </row>
     <row r="10">
       <c r="F10" s="70" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="67" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B11" s="69"/>
       <c r="F11" s="70" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B12" s="2">
         <v>8678212.336123724</v>
       </c>
       <c r="F12" s="70" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B13" s="2">
         <v>520000.0</v>
       </c>
       <c r="F13" s="70" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B14" s="2">
         <v>4920000.0</v>
@@ -6588,7 +6594,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B15" s="71">
         <v>3758212.3361237235</v>
@@ -6600,13 +6606,13 @@
     </row>
     <row r="17">
       <c r="A17" s="67" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B17" s="69"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B18" s="2">
         <v>350000.0</v>
@@ -6614,7 +6620,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B19" s="2">
         <v>7.5E7</v>
@@ -6622,7 +6628,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B20" s="2">
         <v>4920000.0</v>
@@ -6630,7 +6636,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B21" s="2">
         <v>350000.0</v>
@@ -6642,13 +6648,13 @@
     </row>
     <row r="23">
       <c r="A23" s="67" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B23" s="69"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B24" s="2">
         <v>605000.0</v>
@@ -6656,7 +6662,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B25" s="2">
         <v>4920000.0</v>
@@ -6664,7 +6670,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B26" s="2">
         <v>-4315000.0</v>
@@ -6672,7 +6678,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B27" s="2">
         <v>-0.4865809652683807</v>
@@ -6680,13 +6686,13 @@
     </row>
     <row r="29">
       <c r="A29" s="72" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B29" s="73"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B30" s="71">
         <v>853884.2975206611</v>
@@ -6694,7 +6700,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B31" s="71">
         <v>1.3016528925619835E7</v>
@@ -6702,7 +6708,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B32" s="71">
         <v>1.2162644628099175E7</v>
@@ -6710,7 +6716,7 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -36655,13 +36661,13 @@
       <c r="H2" s="57">
         <v>16.0</v>
       </c>
-      <c r="I2" s="27" t="b">
-        <v>1</v>
+      <c r="I2" s="3" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>229</v>
@@ -36670,7 +36676,7 @@
         <v>242</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E3" s="44">
         <v>80000.0</v>
@@ -36684,13 +36690,13 @@
       <c r="H3" s="57">
         <v>1.5</v>
       </c>
-      <c r="I3" s="27" t="b">
-        <v>1</v>
+      <c r="I3" s="3" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>231</v>
@@ -36699,7 +36705,7 @@
         <v>242</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E4" s="44">
         <v>140000.0</v>
@@ -36713,8 +36719,8 @@
       <c r="H4" s="57">
         <v>0.0</v>
       </c>
-      <c r="I4" s="27" t="b">
-        <v>0</v>
+      <c r="I4" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
@@ -36728,8 +36734,8 @@
       <c r="H5" s="57">
         <v>0.0</v>
       </c>
-      <c r="I5" s="27" t="b">
-        <v>0</v>
+      <c r="I5" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
@@ -36743,8 +36749,8 @@
       <c r="H6" s="57">
         <v>0.0</v>
       </c>
-      <c r="I6" s="27" t="b">
-        <v>0</v>
+      <c r="I6" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -36758,8 +36764,8 @@
       <c r="H7" s="57">
         <v>0.0</v>
       </c>
-      <c r="I7" s="27" t="b">
-        <v>0</v>
+      <c r="I7" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
@@ -36773,8 +36779,8 @@
       <c r="H8" s="57">
         <v>0.0</v>
       </c>
-      <c r="I8" s="27" t="b">
-        <v>0</v>
+      <c r="I8" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
@@ -36788,8 +36794,8 @@
       <c r="H9" s="57">
         <v>0.0</v>
       </c>
-      <c r="I9" s="27" t="b">
-        <v>0</v>
+      <c r="I9" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
@@ -36803,8 +36809,8 @@
       <c r="H10" s="57">
         <v>0.0</v>
       </c>
-      <c r="I10" s="27" t="b">
-        <v>0</v>
+      <c r="I10" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
@@ -36818,8 +36824,8 @@
       <c r="H11" s="57">
         <v>0.0</v>
       </c>
-      <c r="I11" s="27" t="b">
-        <v>0</v>
+      <c r="I11" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
@@ -36833,8 +36839,8 @@
       <c r="H12" s="57">
         <v>0.0</v>
       </c>
-      <c r="I12" s="27" t="b">
-        <v>0</v>
+      <c r="I12" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
@@ -36848,8 +36854,8 @@
       <c r="H13" s="57">
         <v>0.0</v>
       </c>
-      <c r="I13" s="27" t="b">
-        <v>0</v>
+      <c r="I13" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
@@ -36863,8 +36869,8 @@
       <c r="H14" s="57">
         <v>0.0</v>
       </c>
-      <c r="I14" s="27" t="b">
-        <v>0</v>
+      <c r="I14" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
@@ -36878,8 +36884,8 @@
       <c r="H15" s="57">
         <v>0.0</v>
       </c>
-      <c r="I15" s="27" t="b">
-        <v>0</v>
+      <c r="I15" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
@@ -36893,8 +36899,8 @@
       <c r="H16" s="57">
         <v>0.0</v>
       </c>
-      <c r="I16" s="27" t="b">
-        <v>0</v>
+      <c r="I16" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
@@ -36908,8 +36914,8 @@
       <c r="H17" s="57">
         <v>0.0</v>
       </c>
-      <c r="I17" s="27" t="b">
-        <v>0</v>
+      <c r="I17" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
@@ -36923,8 +36929,8 @@
       <c r="H18" s="57">
         <v>0.0</v>
       </c>
-      <c r="I18" s="27" t="b">
-        <v>0</v>
+      <c r="I18" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="19">
@@ -39880,6 +39886,9 @@
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="E2:E18">
       <formula1>AND(ISNUMBER(E2),(NOT(OR(NOT(ISERROR(DATEVALUE(E2))), AND(ISNUMBER(E2), LEFT(CELL("format", E2))="D")))))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="I2:I18">
+      <formula1>"Completed,Active"</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>
@@ -39908,7 +39917,7 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>135</v>
@@ -39917,10 +39926,10 @@
         <v>137</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>157</v>
@@ -39932,15 +39941,15 @@
         <v>2</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="J1" s="41" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B2" s="5">
         <v>46133.0</v>
@@ -39967,12 +39976,12 @@
         <v>46065.0</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B3" s="5">
         <v>46134.0</v>
@@ -39984,7 +39993,7 @@
         <v>229</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>168</v>
@@ -39999,12 +40008,12 @@
         <v>46084.0</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B4" s="5">
         <v>46135.0</v>
@@ -40025,18 +40034,18 @@
         <v>100000.0</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="I4" s="5">
         <v>46065.0</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B5" s="5">
         <v>46136.0</v>
@@ -40063,7 +40072,7 @@
         <v>46129.0</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">

</xml_diff>